<commit_message>
Fixing Tennessee state name
</commit_message>
<xml_diff>
--- a/AHR 30th/AHR_data 30th dashboard.xlsx
+++ b/AHR 30th/AHR_data 30th dashboard.xlsx
@@ -16918,13 +16918,13 @@
         <v>1.546558739611991</v>
       </c>
       <c r="G502">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H502">
-        <v>1.343662560004414</v>
+        <v>1.386367951805704</v>
       </c>
       <c r="I502">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="503">
@@ -16951,13 +16951,13 @@
         <v>1.916588853159228</v>
       </c>
       <c r="G503">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H503">
-        <v>1.665147672023079</v>
+        <v>1.718070768831341</v>
       </c>
       <c r="I503">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="504">
@@ -16984,13 +16984,13 @@
         <v>1.437964708203125</v>
       </c>
       <c r="G504">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H504">
-        <v>1.249315199954809</v>
+        <v>1.289021966136641</v>
       </c>
       <c r="I504">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="505">
@@ -17017,13 +17017,13 @@
         <v>1.791750853497073</v>
       </c>
       <c r="G505">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H505">
-        <v>1.556687422880544</v>
+        <v>1.606163346587189</v>
       </c>
       <c r="I505">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="506">
@@ -17050,13 +17050,13 @@
         <v>1.158444012988471</v>
       </c>
       <c r="G506">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H506">
-        <v>1.006465391999526</v>
+        <v>1.03845370527041</v>
       </c>
       <c r="I506">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="507">
@@ -17083,13 +17083,13 @@
         <v>1.323958484081296</v>
       </c>
       <c r="G507">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H507">
-        <v>1.150265683737659</v>
+        <v>1.186824376494145</v>
       </c>
       <c r="I507">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="508">
@@ -17116,10 +17116,10 @@
         <v>0.557401017424077</v>
       </c>
       <c r="G508">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H508">
-        <v>0.484274446768833</v>
+        <v>0.4996660566895171</v>
       </c>
       <c r="I508">
         <v>3</v>
@@ -17149,10 +17149,10 @@
         <v>0.9435103377597176</v>
       </c>
       <c r="G509">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H509">
-        <v>0.8197293018064832</v>
+        <v>0.8457826146297031</v>
       </c>
       <c r="I509">
         <v>18</v>
@@ -17182,13 +17182,13 @@
         <v>1.54518544526613</v>
       </c>
       <c r="G510">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H510">
-        <v>1.342469430930725</v>
+        <v>1.385136901719643</v>
       </c>
       <c r="I510">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="511">
@@ -17215,10 +17215,10 @@
         <v>0.8306768720704029</v>
       </c>
       <c r="G511">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H511">
-        <v>0.7216986874631109</v>
+        <v>0.7446363104407784</v>
       </c>
       <c r="I511">
         <v>13</v>
@@ -17248,13 +17248,13 @@
         <v>3.143211060938769</v>
       </c>
       <c r="G512">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H512">
-        <v>2.730846823079459</v>
+        <v>2.817640849347879</v>
       </c>
       <c r="I512">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="513">
@@ -17281,13 +17281,13 @@
         <v>1.424057155134427</v>
       </c>
       <c r="G513">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H513">
-        <v>1.237232206996926</v>
+        <v>1.276554941529921</v>
       </c>
       <c r="I513">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="514">
@@ -17314,10 +17314,10 @@
         <v>0.9563043256849029</v>
       </c>
       <c r="G514">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H514">
-        <v>0.8308448204918795</v>
+        <v>0.8572514158985873</v>
       </c>
       <c r="I514">
         <v>20</v>
@@ -17347,13 +17347,13 @@
         <v>1.042099344822047</v>
       </c>
       <c r="G515">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H515">
-        <v>0.9053842169575864</v>
+        <v>0.9341598849465423</v>
       </c>
       <c r="I515">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="516">
@@ -17380,10 +17380,10 @@
         <v>0.64135605439773</v>
       </c>
       <c r="G516">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H516">
-        <v>0.5572152520651036</v>
+        <v>0.5749251268248918</v>
       </c>
       <c r="I516">
         <v>8</v>
@@ -17413,10 +17413,10 @@
         <v>0.9315724843391602</v>
       </c>
       <c r="G517">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H517">
-        <v>0.809357599602629</v>
+        <v>0.8350812704313139</v>
       </c>
       <c r="I517">
         <v>17</v>
@@ -17446,13 +17446,13 @@
         <v>1.023625905976862</v>
       </c>
       <c r="G518">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H518">
-        <v>0.8893343460441584</v>
+        <v>0.9175999037970177</v>
       </c>
       <c r="I518">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="519">
@@ -17479,13 +17479,13 @@
         <v>0.9691454880831557</v>
       </c>
       <c r="G519">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H519">
-        <v>0.8420013247354865</v>
+        <v>0.8687625053625003</v>
       </c>
       <c r="I519">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="520">
@@ -17512,13 +17512,13 @@
         <v>1.077728692938083</v>
       </c>
       <c r="G520">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H520">
-        <v>0.9363392785887356</v>
+        <v>0.9660987858797161</v>
       </c>
       <c r="I520">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="521">
@@ -17545,10 +17545,10 @@
         <v>0.5978690522960789</v>
       </c>
       <c r="G521">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H521">
-        <v>0.5194333980208908</v>
+        <v>0.535942458731107</v>
       </c>
       <c r="I521">
         <v>7</v>
@@ -17578,10 +17578,10 @@
         <v>0.7424728473967344</v>
       </c>
       <c r="G522">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H522">
-        <v>0.6450663277860074</v>
+        <v>0.6655683578982627</v>
       </c>
       <c r="I522">
         <v>11</v>
@@ -17611,10 +17611,10 @@
         <v>0.8125484229061878</v>
       </c>
       <c r="G523">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H523">
-        <v>0.7059485463342907</v>
+        <v>0.7283855853351079</v>
       </c>
       <c r="I523">
         <v>12</v>
@@ -17644,10 +17644,10 @@
         <v>0.8978072570646936</v>
       </c>
       <c r="G524">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H524">
-        <v>0.7800221010168312</v>
+        <v>0.8048134068320945</v>
       </c>
       <c r="I524">
         <v>15</v>
@@ -17677,13 +17677,13 @@
         <v>1.652932463280736</v>
       </c>
       <c r="G525">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H525">
-        <v>1.436080898992177</v>
+        <v>1.481723606674385</v>
       </c>
       <c r="I525">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="526">
@@ -17710,13 +17710,13 @@
         <v>1.038530651512329</v>
       </c>
       <c r="G526">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H526">
-        <v>0.9022837077654113</v>
+        <v>0.9309608328137686</v>
       </c>
       <c r="I526">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="527">
@@ -17743,13 +17743,13 @@
         <v>1.265166521633523</v>
       </c>
       <c r="G527">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H527">
-        <v>1.099186758154736</v>
+        <v>1.134122018365926</v>
       </c>
       <c r="I527">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="528">
@@ -17776,13 +17776,13 @@
         <v>1.158331431633449</v>
       </c>
       <c r="G528">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H528">
-        <v>1.00636758042094</v>
+        <v>1.038352784963554</v>
       </c>
       <c r="I528">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="529">
@@ -17809,13 +17809,13 @@
         <v>1.331149152665648</v>
       </c>
       <c r="G529">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H529">
-        <v>1.156512993917818</v>
+        <v>1.19327024383954</v>
       </c>
       <c r="I529">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="530">
@@ -17842,10 +17842,10 @@
         <v>0.8989784599538359</v>
       </c>
       <c r="G530">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H530">
-        <v>0.7810396514221293</v>
+        <v>0.8058632978636996</v>
       </c>
       <c r="I530">
         <v>16</v>
@@ -17875,13 +17875,13 @@
         <v>1.757109056582949</v>
       </c>
       <c r="G531">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H531">
-        <v>1.526590353605009</v>
+        <v>1.57510970743039</v>
       </c>
       <c r="I531">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="532">
@@ -17908,13 +17908,13 @@
         <v>1.621249915389613</v>
       </c>
       <c r="G532">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H532">
-        <v>1.408554848854871</v>
+        <v>1.45332270090677</v>
       </c>
       <c r="I532">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="533">
@@ -17941,10 +17941,10 @@
         <v>0.5653356515936899</v>
       </c>
       <c r="G533">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H533">
-        <v>0.4911681201793336</v>
+        <v>0.5067788305145926</v>
       </c>
       <c r="I533">
         <v>4</v>
@@ -17974,13 +17974,13 @@
         <v>1.176656778823377</v>
       </c>
       <c r="G534">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H534">
-        <v>1.022288788123899</v>
+        <v>1.054780013622326</v>
       </c>
       <c r="I534">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="535">
@@ -18007,10 +18007,10 @@
         <v>0.8899499884751475</v>
       </c>
       <c r="G535">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H535">
-        <v>0.7731956434389442</v>
+        <v>0.7977699851486677</v>
       </c>
       <c r="I535">
         <v>14</v>
@@ -18040,10 +18040,10 @@
         <v>0.6690928544011803</v>
       </c>
       <c r="G536">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H536">
-        <v>0.5813132049875491</v>
+        <v>0.5997889807643001</v>
       </c>
       <c r="I536">
         <v>9</v>
@@ -18073,10 +18073,10 @@
         <v>0.9574745409619284</v>
       </c>
       <c r="G537">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H537">
-        <v>0.8318615128518986</v>
+        <v>0.8583004216138107</v>
       </c>
       <c r="I537">
         <v>21</v>
@@ -18106,13 +18106,13 @@
         <v>1.674049694553563</v>
       </c>
       <c r="G538">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H538">
-        <v>1.454427717839401</v>
+        <v>1.500653539251574</v>
       </c>
       <c r="I538">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="539">
@@ -18139,10 +18139,10 @@
         <v>0.5812995077504219</v>
       </c>
       <c r="G539">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H539">
-        <v>0.5050376456501077</v>
+        <v>0.5210891686841483</v>
       </c>
       <c r="I539">
         <v>6</v>
@@ -18172,10 +18172,10 @@
         <v>0.5727315192711556</v>
       </c>
       <c r="G540">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H540">
-        <v>0.4975937089671547</v>
+        <v>0.5134086426654111</v>
       </c>
       <c r="I540">
         <v>5</v>
@@ -18205,13 +18205,13 @@
         <v>1.732935271076938</v>
       </c>
       <c r="G541">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H541">
-        <v>1.505587976077368</v>
+        <v>1.553439815016368</v>
       </c>
       <c r="I541">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="542">
@@ -18238,13 +18238,13 @@
         <v>1.075570109353639</v>
       </c>
       <c r="G542">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H542">
-        <v>0.9344638839653246</v>
+        <v>0.9641637859174659</v>
       </c>
       <c r="I542">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="543">
@@ -18259,13 +18259,25 @@
       <c r="C543">
         <v>156</v>
       </c>
+      <c r="D543">
+        <v>16164.75063</v>
+      </c>
       <c r="E543" t="inlineStr">
         <is>
           <t>rural_fatalities_per_100m_VMT_score</t>
         </is>
       </c>
+      <c r="F543">
+        <v>0.9650628306661357</v>
+      </c>
       <c r="G543">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
+      </c>
+      <c r="H543">
+        <v>0.8651027249376209</v>
+      </c>
+      <c r="I543">
+        <v>22</v>
       </c>
     </row>
     <row r="544">
@@ -18292,13 +18304,13 @@
         <v>1.337922335752768</v>
       </c>
       <c r="G544">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H544">
-        <v>1.162397589370366</v>
+        <v>1.199341868358666</v>
       </c>
       <c r="I544">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="545">
@@ -18325,13 +18337,13 @@
         <v>1.180604144687008</v>
       </c>
       <c r="G545">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H545">
-        <v>1.025718291049169</v>
+        <v>1.05831851583839</v>
       </c>
       <c r="I545">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="546">
@@ -18358,10 +18370,10 @@
         <v>0.5408658706973106</v>
       </c>
       <c r="G546">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H546">
-        <v>0.4699085794972739</v>
+        <v>0.4848436015746567</v>
       </c>
       <c r="I546">
         <v>2</v>
@@ -18391,13 +18403,13 @@
         <v>1.25354972894032</v>
       </c>
       <c r="G547">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H547">
-        <v>1.089093996069861</v>
+        <v>1.12370847979146</v>
       </c>
       <c r="I547">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="548">
@@ -18424,13 +18436,13 @@
         <v>1.053732927431458</v>
       </c>
       <c r="G548">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H548">
-        <v>0.9154915662554906</v>
+        <v>0.9445884743568733</v>
       </c>
       <c r="I548">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="549">
@@ -18457,10 +18469,10 @@
         <v>0.711916799512206</v>
       </c>
       <c r="G549">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H549">
-        <v>0.6185189898333322</v>
+        <v>0.6381772705532205</v>
       </c>
       <c r="I549">
         <v>10</v>
@@ -18490,10 +18502,10 @@
         <v>0.4906469365723513</v>
       </c>
       <c r="G550">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H550">
-        <v>0.4262779692535499</v>
+        <v>0.4398262872874848</v>
       </c>
       <c r="I550">
         <v>1</v>
@@ -18523,10 +18535,10 @@
         <v>0.9495847396975362</v>
       </c>
       <c r="G551">
-        <v>1.151002331721522</v>
+        <v>1.115547093827178</v>
       </c>
       <c r="H551">
-        <v>0.8250067906267997</v>
+        <v>0.8512278369528403</v>
       </c>
       <c r="I551">
         <v>19</v>
@@ -18556,10 +18568,10 @@
         <v>1.061679741146842</v>
       </c>
       <c r="G552">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H552">
-        <v>1.105390411122654</v>
+        <v>1.132780640519556</v>
       </c>
       <c r="I552">
         <v>36</v>
@@ -18589,10 +18601,10 @@
         <v>1.261411418464348</v>
       </c>
       <c r="G553">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H553">
-        <v>1.313345288989801</v>
+        <v>1.345888387229848</v>
       </c>
       <c r="I553">
         <v>45</v>
@@ -18622,10 +18634,10 @@
         <v>1.23537942968035</v>
       </c>
       <c r="G554">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H554">
-        <v>1.286241530983455</v>
+        <v>1.318113031078773</v>
       </c>
       <c r="I554">
         <v>43</v>
@@ -18655,10 +18667,10 @@
         <v>0.9822082835756718</v>
       </c>
       <c r="G555">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H555">
-        <v>1.022647015207217</v>
+        <v>1.04798696393188</v>
       </c>
       <c r="I555">
         <v>26</v>
@@ -18688,10 +18700,10 @@
         <v>0.9125068253040979</v>
       </c>
       <c r="G556">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H556">
-        <v>0.9500758615639947</v>
+        <v>0.9736175854027854</v>
       </c>
       <c r="I556">
         <v>23</v>
@@ -18721,10 +18733,10 @@
         <v>1.191299959746605</v>
       </c>
       <c r="G557">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H557">
-        <v>1.240347254674201</v>
+        <v>1.271081550444724</v>
       </c>
       <c r="I557">
         <v>41</v>
@@ -18754,10 +18766,10 @@
         <v>0.7196827190122299</v>
       </c>
       <c r="G558">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H558">
-        <v>0.7493129479775652</v>
+        <v>0.7678800110972188</v>
       </c>
       <c r="I558">
         <v>19</v>
@@ -18787,10 +18799,10 @@
         <v>0.9913191410168661</v>
       </c>
       <c r="G559">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H559">
-        <v>1.032132977934284</v>
+        <v>1.05770797727322</v>
       </c>
       <c r="I559">
         <v>27</v>
@@ -18820,10 +18832,10 @@
         <v>1.175569279528065</v>
       </c>
       <c r="G560">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H560">
-        <v>1.223968922866506</v>
+        <v>1.254297383503272</v>
       </c>
       <c r="I560">
         <v>39</v>
@@ -18853,10 +18865,10 @@
         <v>1.031157054593156</v>
       </c>
       <c r="G561">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H561">
-        <v>1.073611067757111</v>
+        <v>1.100213843693129</v>
       </c>
       <c r="I561">
         <v>32</v>
@@ -18886,10 +18898,10 @@
         <v>1.143791676866334</v>
       </c>
       <c r="G562">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H562">
-        <v>1.190882996942366</v>
+        <v>1.22039162859224</v>
       </c>
       <c r="I562">
         <v>38</v>
@@ -18919,10 +18931,10 @@
         <v>0.6697451321627513</v>
       </c>
       <c r="G563">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H563">
-        <v>0.6973193688230925</v>
+        <v>0.7145980943148119</v>
       </c>
       <c r="I563">
         <v>11</v>
@@ -18952,10 +18964,10 @@
         <v>0.9713350183635551</v>
       </c>
       <c r="G564">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H564">
-        <v>1.011326084198319</v>
+        <v>1.036385514027396</v>
       </c>
       <c r="I564">
         <v>25</v>
@@ -18985,10 +18997,10 @@
         <v>0.6881759063033738</v>
       </c>
       <c r="G565">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H565">
-        <v>0.7165089607640709</v>
+        <v>0.7342631809950314</v>
       </c>
       <c r="I565">
         <v>16</v>
@@ -19018,10 +19030,10 @@
         <v>0.6477854046018922</v>
       </c>
       <c r="G566">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H566">
-        <v>0.6744555320784841</v>
+        <v>0.6911677195153888</v>
       </c>
       <c r="I566">
         <v>10</v>
@@ -19051,10 +19063,10 @@
         <v>0.6714571986417301</v>
       </c>
       <c r="G567">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H567">
-        <v>0.6991019231996349</v>
+        <v>0.7164248182198708</v>
       </c>
       <c r="I567">
         <v>13</v>
@@ -19084,10 +19096,10 @@
         <v>0.9664382251635665</v>
       </c>
       <c r="G568">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H568">
-        <v>1.006227683956952</v>
+        <v>1.031160781631558</v>
       </c>
       <c r="I568">
         <v>24</v>
@@ -19117,10 +19129,10 @@
         <v>1.199541949337344</v>
       </c>
       <c r="G569">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H569">
-        <v>1.2489285771852</v>
+        <v>1.279875507686167</v>
       </c>
       <c r="I569">
         <v>42</v>
@@ -19150,10 +19162,10 @@
         <v>0.5028678933106425</v>
       </c>
       <c r="G570">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H570">
-        <v>0.5235715873475935</v>
+        <v>0.5365450542230532</v>
       </c>
       <c r="I570">
         <v>3</v>
@@ -19183,10 +19195,10 @@
         <v>1.011113274179578</v>
       </c>
       <c r="G571">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H571">
-        <v>1.052742060076994</v>
+        <v>1.078827727395196</v>
       </c>
       <c r="I571">
         <v>28</v>
@@ -19216,10 +19228,10 @@
         <v>0.5233313811194925</v>
       </c>
       <c r="G572">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H572">
-        <v>0.5448775822963089</v>
+        <v>0.5583789858023948</v>
       </c>
       <c r="I572">
         <v>6</v>
@@ -19249,10 +19261,10 @@
         <v>0.8461012176731455</v>
       </c>
       <c r="G573">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H573">
-        <v>0.8809362528146218</v>
+        <v>0.9027647812746559</v>
       </c>
       <c r="I573">
         <v>21</v>
@@ -19282,10 +19294,10 @@
         <v>0.3507276065045727</v>
       </c>
       <c r="G574">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H574">
-        <v>0.3651674964875611</v>
+        <v>0.3742159027306805</v>
       </c>
       <c r="I574">
         <v>2</v>
@@ -19315,13 +19327,13 @@
         <v>1.500817967161366</v>
       </c>
       <c r="G575">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H575">
-        <v>1.562608501833805</v>
+        <v>1.601328039195548</v>
       </c>
       <c r="I575">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="576">
@@ -19348,10 +19360,10 @@
         <v>1.023679431315542</v>
       </c>
       <c r="G576">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H576">
-        <v>1.065825581467118</v>
+        <v>1.09223544252591</v>
       </c>
       <c r="I576">
         <v>31</v>
@@ -19381,13 +19393,13 @@
         <v>1.446432915893151</v>
       </c>
       <c r="G577">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H577">
-        <v>1.505984350641695</v>
+        <v>1.543300810434689</v>
       </c>
       <c r="I577">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="578">
@@ -19414,10 +19426,10 @@
         <v>0.7859966683846932</v>
       </c>
       <c r="G578">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H578">
-        <v>0.8183571247844159</v>
+        <v>0.838635018595408</v>
       </c>
       <c r="I578">
         <v>20</v>
@@ -19447,10 +19459,10 @@
         <v>1.182648816398851</v>
       </c>
       <c r="G579">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H579">
-        <v>1.231339933039217</v>
+        <v>1.26185103833934</v>
       </c>
       <c r="I579">
         <v>40</v>
@@ -19480,10 +19492,10 @@
         <v>0.6796333690605267</v>
       </c>
       <c r="G580">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H580">
-        <v>0.7076147166818574</v>
+        <v>0.7251485483665879</v>
       </c>
       <c r="I580">
         <v>14</v>
@@ -19513,10 +19525,10 @@
         <v>0.700370091056468</v>
       </c>
       <c r="G581">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H581">
-        <v>0.7292051952075838</v>
+        <v>0.7472740126798316</v>
       </c>
       <c r="I581">
         <v>17</v>
@@ -19546,13 +19558,13 @@
         <v>1.38842927040198</v>
       </c>
       <c r="G582">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H582">
-        <v>1.445592623220356</v>
+        <v>1.481412649489863</v>
       </c>
       <c r="I582">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="583">
@@ -19579,10 +19591,10 @@
         <v>0.7028487842852077</v>
       </c>
       <c r="G583">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H583">
-        <v>0.7317859393067448</v>
+        <v>0.7499187044776333</v>
       </c>
       <c r="I583">
         <v>18</v>
@@ -19612,10 +19624,10 @@
         <v>0.891645867969482</v>
       </c>
       <c r="G584">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H584">
-        <v>0.9283560327768183</v>
+        <v>0.9513595656860007</v>
       </c>
       <c r="I584">
         <v>22</v>
@@ -19645,10 +19657,10 @@
         <v>0.3302821603137818</v>
       </c>
       <c r="G585">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H585">
-        <v>0.3438802859526671</v>
+        <v>0.3524012210200789</v>
       </c>
       <c r="I585">
         <v>1</v>
@@ -19678,10 +19690,10 @@
         <v>0.687999405488645</v>
       </c>
       <c r="G586">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H586">
-        <v>0.7163251931921798</v>
+        <v>0.7340748598863092</v>
       </c>
       <c r="I586">
         <v>15</v>
@@ -19711,10 +19723,10 @@
         <v>1.072860645259916</v>
       </c>
       <c r="G587">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H587">
-        <v>1.117031646907113</v>
+        <v>1.144710331962207</v>
       </c>
       <c r="I587">
         <v>37</v>
@@ -19744,10 +19756,10 @@
         <v>1.040451958710402</v>
       </c>
       <c r="G588">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H588">
-        <v>1.083288654589849</v>
+        <v>1.110131229352319</v>
       </c>
       <c r="I588">
         <v>34</v>
@@ -19777,10 +19789,10 @@
         <v>1.01980536865182</v>
       </c>
       <c r="G589">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H589">
-        <v>1.061792018844983</v>
+        <v>1.088101933129862</v>
       </c>
       <c r="I589">
         <v>30</v>
@@ -19810,10 +19822,10 @@
         <v>0.5037562395090401</v>
       </c>
       <c r="G590">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H590">
-        <v>0.524496507859315</v>
+        <v>0.5374928931396524</v>
       </c>
       <c r="I590">
         <v>4</v>
@@ -19843,13 +19855,13 @@
         <v>1.310287011813789</v>
       </c>
       <c r="G591">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H591">
-        <v>1.364233151056419</v>
+        <v>1.398037188600351</v>
       </c>
       <c r="I591">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="592">
@@ -19876,10 +19888,10 @@
         <v>0.5195600425309252</v>
       </c>
       <c r="G592">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H592">
-        <v>0.5409509730267414</v>
+        <v>0.5543550799328539</v>
       </c>
       <c r="I592">
         <v>5</v>
@@ -19897,13 +19909,25 @@
       <c r="C593">
         <v>415</v>
       </c>
+      <c r="D593">
+        <v>31959.74724</v>
+      </c>
       <c r="E593" t="inlineStr">
         <is>
           <t>urban_fatalities_per_100m_VMT_score</t>
         </is>
       </c>
+      <c r="F593">
+        <v>1.298508392083266</v>
+      </c>
       <c r="G593">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
+      </c>
+      <c r="H593">
+        <v>1.38546975240875</v>
+      </c>
+      <c r="I593">
+        <v>46</v>
       </c>
     </row>
     <row r="594">
@@ -19930,10 +19954,10 @@
         <v>1.033397367658967</v>
       </c>
       <c r="G594">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H594">
-        <v>1.075943617286769</v>
+        <v>1.102604190961989</v>
       </c>
       <c r="I594">
         <v>33</v>
@@ -19963,10 +19987,10 @@
         <v>0.5521000077874636</v>
       </c>
       <c r="G595">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H595">
-        <v>0.5748306489580042</v>
+        <v>0.589074253010385</v>
       </c>
       <c r="I595">
         <v>7</v>
@@ -19996,10 +20020,10 @@
         <v>0.5689224355899444</v>
       </c>
       <c r="G596">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H596">
-        <v>0.5923456769499468</v>
+        <v>0.6070232820844478</v>
       </c>
       <c r="I596">
         <v>8</v>
@@ -20029,10 +20053,10 @@
         <v>0.6701119199469469</v>
       </c>
       <c r="G597">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H597">
-        <v>0.6977012577146793</v>
+        <v>0.7149894459484665</v>
       </c>
       <c r="I597">
         <v>12</v>
@@ -20062,10 +20086,10 @@
         <v>1.016886976352176</v>
       </c>
       <c r="G598">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H598">
-        <v>1.058753472719543</v>
+        <v>1.084988095528603</v>
       </c>
       <c r="I598">
         <v>29</v>
@@ -20095,10 +20119,10 @@
         <v>1.238794342396874</v>
       </c>
       <c r="G599">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H599">
-        <v>1.289797039886346</v>
+        <v>1.32175664116609</v>
       </c>
       <c r="I599">
         <v>44</v>
@@ -20128,10 +20152,10 @@
         <v>0.6403066259390674</v>
       </c>
       <c r="G600">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H600">
-        <v>0.66666884283464</v>
+        <v>0.6831880855865854</v>
       </c>
       <c r="I600">
         <v>9</v>
@@ -20161,10 +20185,10 @@
         <v>1.051504159876637</v>
       </c>
       <c r="G601">
-        <v>0.9604568037355969</v>
+        <v>0.9372333028748592</v>
       </c>
       <c r="H601">
-        <v>1.094795888567732</v>
+        <v>1.121923598586675</v>
       </c>
       <c r="I601">
         <v>35</v>
@@ -20194,10 +20218,10 @@
         <v>1.376907820757462</v>
       </c>
       <c r="G602">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H602">
-        <v>0.950295253754483</v>
+        <v>0.9709932027434547</v>
       </c>
       <c r="I602">
         <v>29</v>
@@ -20227,10 +20251,10 @@
         <v>0.9856966282590103</v>
       </c>
       <c r="G603">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H603">
-        <v>0.6802945072684946</v>
+        <v>0.6951116927203739</v>
       </c>
       <c r="I603">
         <v>7</v>
@@ -20260,13 +20284,13 @@
         <v>2.124589567809786</v>
       </c>
       <c r="G604">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H604">
-        <v>1.466319932263327</v>
+        <v>1.498257180228726</v>
       </c>
       <c r="I604">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="605">
@@ -20293,10 +20317,10 @@
         <v>1.729944927007016</v>
       </c>
       <c r="G605">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H605">
-        <v>1.19394953576997</v>
+        <v>1.219954407928531</v>
       </c>
       <c r="I605">
         <v>42</v>
@@ -20326,10 +20350,10 @@
         <v>1.657149781407989</v>
       </c>
       <c r="G606">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H606">
-        <v>1.143708785941803</v>
+        <v>1.16861938716404</v>
       </c>
       <c r="I606">
         <v>39</v>
@@ -20359,10 +20383,10 @@
         <v>1.291920192878279</v>
       </c>
       <c r="G607">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H607">
-        <v>0.8916396646265115</v>
+        <v>0.9110600628891249</v>
       </c>
       <c r="I607">
         <v>18</v>
@@ -20392,10 +20416,10 @@
         <v>1.453119341995307</v>
       </c>
       <c r="G608">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H608">
-        <v>1.002893870613157</v>
+        <v>1.024737446168535</v>
       </c>
       <c r="I608">
         <v>32</v>
@@ -20425,10 +20449,10 @@
         <v>1.619642869533952</v>
       </c>
       <c r="G609">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H609">
-        <v>1.117822782681775</v>
+        <v>1.142169572632844</v>
       </c>
       <c r="I609">
         <v>37</v>
@@ -20458,10 +20482,10 @@
         <v>1.192460724106906</v>
       </c>
       <c r="G610">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H610">
-        <v>0.8229960999016175</v>
+        <v>0.8409214038811818</v>
       </c>
       <c r="I610">
         <v>14</v>
@@ -20491,10 +20515,10 @@
         <v>1.331335669055292</v>
       </c>
       <c r="G611">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H611">
-        <v>0.9188428944802592</v>
+        <v>0.9388557939277661</v>
       </c>
       <c r="I611">
         <v>24</v>
@@ -20524,10 +20548,10 @@
         <v>0.6786476065228866</v>
       </c>
       <c r="G612">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H612">
-        <v>0.4683796472996711</v>
+        <v>0.4785812115071946</v>
       </c>
       <c r="I612">
         <v>2</v>
@@ -20557,10 +20581,10 @@
         <v>1.293098669726099</v>
       </c>
       <c r="G613">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H613">
-        <v>0.8924530095274993</v>
+        <v>0.9118911228857154</v>
       </c>
       <c r="I613">
         <v>19</v>
@@ -20590,10 +20614,10 @@
         <v>1.322136431171046</v>
       </c>
       <c r="G614">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H614">
-        <v>0.9124938913242251</v>
+        <v>0.9323685060197717</v>
       </c>
       <c r="I614">
         <v>22</v>
@@ -20623,10 +20647,10 @@
         <v>1.028614968017167</v>
       </c>
       <c r="G615">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H615">
-        <v>0.7099152952082147</v>
+        <v>0.7253776375788172</v>
       </c>
       <c r="I615">
         <v>10</v>
@@ -20656,10 +20680,10 @@
         <v>1.583484806397701</v>
       </c>
       <c r="G616">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H616">
-        <v>1.09286770924452</v>
+        <v>1.116670964083759</v>
       </c>
       <c r="I616">
         <v>34</v>
@@ -20689,10 +20713,10 @@
         <v>1.319627999780003</v>
       </c>
       <c r="G617">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H617">
-        <v>0.9107626567351403</v>
+        <v>0.9305995641969917</v>
       </c>
       <c r="I617">
         <v>21</v>
@@ -20722,10 +20746,10 @@
         <v>1.942203917118805</v>
       </c>
       <c r="G618">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H618">
-        <v>1.340443518757872</v>
+        <v>1.369639109774699</v>
       </c>
       <c r="I618">
         <v>46</v>
@@ -20755,10 +20779,10 @@
         <v>1.613310347190545</v>
       </c>
       <c r="G619">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H619">
-        <v>1.113452289729006</v>
+        <v>1.137703887959569</v>
       </c>
       <c r="I619">
         <v>36</v>
@@ -20788,10 +20812,10 @@
         <v>1.374254424733155</v>
       </c>
       <c r="G620">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H620">
-        <v>0.9484639694737076</v>
+        <v>0.9691220320921243</v>
       </c>
       <c r="I620">
         <v>28</v>
@@ -20821,10 +20845,10 @@
         <v>1.116408646892007</v>
       </c>
       <c r="G621">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H621">
-        <v>0.7705075259201506</v>
+        <v>0.7872896001271995</v>
       </c>
       <c r="I621">
         <v>12</v>
@@ -20854,10 +20878,10 @@
         <v>0.6589473424623987</v>
       </c>
       <c r="G622">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H622">
-        <v>0.4547831906943969</v>
+        <v>0.4646886166605317</v>
       </c>
       <c r="I622">
         <v>1</v>
@@ -20887,10 +20911,10 @@
         <v>1.367814752575387</v>
       </c>
       <c r="G623">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H623">
-        <v>0.944019525339535</v>
+        <v>0.9645807855403769</v>
       </c>
       <c r="I623">
         <v>27</v>
@@ -20920,10 +20944,10 @@
         <v>0.9749327334081804</v>
       </c>
       <c r="G624">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H624">
-        <v>0.6728656307420843</v>
+        <v>0.6875210112109528</v>
       </c>
       <c r="I624">
         <v>6</v>
@@ -20953,10 +20977,10 @@
         <v>1.885996081543883</v>
       </c>
       <c r="G625">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H625">
-        <v>1.301650769842206</v>
+        <v>1.330001433627179</v>
       </c>
       <c r="I625">
         <v>43</v>
@@ -20986,10 +21010,10 @@
         <v>1.016119235271226</v>
       </c>
       <c r="G626">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H626">
-        <v>0.7012911626834096</v>
+        <v>0.7165656667433741</v>
       </c>
       <c r="I626">
         <v>9</v>
@@ -21019,10 +21043,10 @@
         <v>1.685846434514267</v>
       </c>
       <c r="G627">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H627">
-        <v>1.163514246288838</v>
+        <v>1.188856221240815</v>
       </c>
       <c r="I627">
         <v>40</v>
@@ -21052,10 +21076,10 @@
         <v>1.326307566181995</v>
       </c>
       <c r="G628">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H628">
-        <v>0.9153726677709252</v>
+        <v>0.9353099837877813</v>
       </c>
       <c r="I628">
         <v>23</v>
@@ -21085,10 +21109,10 @@
         <v>1.45342616195017</v>
       </c>
       <c r="G629">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H629">
-        <v>1.00310562737891</v>
+        <v>1.024953815112154</v>
       </c>
       <c r="I629">
         <v>33</v>
@@ -21118,10 +21142,10 @@
         <v>1.197246280140075</v>
       </c>
       <c r="G630">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H630">
-        <v>0.8262989289772738</v>
+        <v>0.8442961703757161</v>
       </c>
       <c r="I630">
         <v>16</v>
@@ -21151,10 +21175,10 @@
         <v>0.9487930017384785</v>
       </c>
       <c r="G631">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H631">
-        <v>0.6548248711751378</v>
+        <v>0.6690873140598569</v>
       </c>
       <c r="I631">
         <v>5</v>
@@ -21184,10 +21208,10 @@
         <v>1.312811911777458</v>
       </c>
       <c r="G632">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H632">
-        <v>0.9060584231035613</v>
+        <v>0.9257928697908755</v>
       </c>
       <c r="I632">
         <v>20</v>
@@ -21217,10 +21241,10 @@
         <v>1.194541570937952</v>
       </c>
       <c r="G633">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H633">
-        <v>0.8244322300749829</v>
+        <v>0.842388813753096</v>
       </c>
       <c r="I633">
         <v>15</v>
@@ -21250,10 +21274,10 @@
         <v>1.429086850448325</v>
       </c>
       <c r="G634">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H634">
-        <v>0.98630745697769</v>
+        <v>1.007789771396616</v>
       </c>
       <c r="I634">
         <v>30</v>
@@ -21283,10 +21307,10 @@
         <v>1.086157823037984</v>
       </c>
       <c r="G635">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H635">
-        <v>0.7496294294366646</v>
+        <v>0.7659567673138257</v>
       </c>
       <c r="I635">
         <v>11</v>
@@ -21316,10 +21340,10 @@
         <v>1.346999624977847</v>
       </c>
       <c r="G636">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H636">
-        <v>0.9296536275909441</v>
+        <v>0.9499019907025851</v>
       </c>
       <c r="I636">
         <v>26</v>
@@ -21349,10 +21373,10 @@
         <v>1.892020534142045</v>
       </c>
       <c r="G637">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H637">
-        <v>1.30580864346613</v>
+        <v>1.334249868006648</v>
       </c>
       <c r="I637">
         <v>44</v>
@@ -21382,10 +21406,10 @@
         <v>1.625212381849401</v>
       </c>
       <c r="G638">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H638">
-        <v>1.12166667189448</v>
+        <v>1.146097183849346</v>
       </c>
       <c r="I638">
         <v>38</v>
@@ -21415,10 +21439,10 @@
         <v>1.603578005470747</v>
       </c>
       <c r="G639">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H639">
-        <v>1.10673535631864</v>
+        <v>1.130840656075606</v>
       </c>
       <c r="I639">
         <v>35</v>
@@ -21448,10 +21472,10 @@
         <v>0.9291123786127875</v>
       </c>
       <c r="G640">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H640">
-        <v>0.6412419700794157</v>
+        <v>0.6552085699691385</v>
       </c>
       <c r="I640">
         <v>4</v>
@@ -21481,10 +21505,10 @@
         <v>1.911937498862678</v>
       </c>
       <c r="G641">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H641">
-        <v>1.319554659544971</v>
+        <v>1.348295279813793</v>
       </c>
       <c r="I641">
         <v>45</v>
@@ -21514,10 +21538,10 @@
         <v>2.023549657207091</v>
       </c>
       <c r="G642">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H642">
-        <v>1.396585599987767</v>
+        <v>1.427003996157877</v>
       </c>
       <c r="I642">
         <v>47</v>
@@ -21535,13 +21559,25 @@
       <c r="C643">
         <v>625</v>
       </c>
+      <c r="D643">
+        <v>30779.92565</v>
+      </c>
       <c r="E643" t="inlineStr">
         <is>
           <t>other_fatalities_per_100m_VMT_score</t>
         </is>
       </c>
+      <c r="F643">
+        <v>2.030544216080652</v>
+      </c>
       <c r="G643">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
+      </c>
+      <c r="H643">
+        <v>1.431936547938054</v>
+      </c>
+      <c r="I643">
+        <v>48</v>
       </c>
     </row>
     <row r="644">
@@ -21568,10 +21604,10 @@
         <v>1.722212539357844</v>
       </c>
       <c r="G644">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H644">
-        <v>1.188612903083</v>
+        <v>1.214501540470641</v>
       </c>
       <c r="I644">
         <v>41</v>
@@ -21601,10 +21637,10 @@
         <v>0.8086699302884396</v>
       </c>
       <c r="G645">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H645">
-        <v>0.5581166618578144</v>
+        <v>0.5702727471917024</v>
       </c>
       <c r="I645">
         <v>3</v>
@@ -21634,10 +21670,10 @@
         <v>0.9951797232199359</v>
       </c>
       <c r="G646">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H646">
-        <v>0.6868394189876488</v>
+        <v>0.7017991561868563</v>
       </c>
       <c r="I646">
         <v>8</v>
@@ -21667,10 +21703,10 @@
         <v>1.332223226835592</v>
       </c>
       <c r="G647">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H647">
-        <v>0.9194554568706659</v>
+        <v>0.9394816982611732</v>
       </c>
       <c r="I647">
         <v>25</v>
@@ -21700,10 +21736,10 @@
         <v>1.452483884490658</v>
       </c>
       <c r="G648">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H648">
-        <v>1.002455299314826</v>
+        <v>1.024289322548097</v>
       </c>
       <c r="I648">
         <v>31</v>
@@ -21733,13 +21769,13 @@
         <v>2.078509820622562</v>
       </c>
       <c r="G649">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H649">
-        <v>1.434517247736388</v>
+        <v>1.465761815885224</v>
       </c>
       <c r="I649">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="650">
@@ -21766,10 +21802,10 @@
         <v>1.176024938556992</v>
       </c>
       <c r="G650">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H650">
-        <v>0.8116526760613654</v>
+        <v>0.8293309140821361</v>
       </c>
       <c r="I650">
         <v>13</v>
@@ -21799,10 +21835,10 @@
         <v>1.266123223323891</v>
       </c>
       <c r="G651">
-        <v>1.44892633664905</v>
+        <v>1.418040638046829</v>
       </c>
       <c r="H651">
-        <v>0.8738354678900174</v>
+        <v>0.8928680810359678</v>
       </c>
       <c r="I651">
         <v>17</v>
@@ -22949,7 +22985,7 @@
         <v>9</v>
       </c>
       <c r="N2">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O2">
         <v>36</v>
@@ -23001,7 +23037,7 @@
         <v>36</v>
       </c>
       <c r="N3">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="O3">
         <v>45</v>
@@ -23020,7 +23056,7 @@
         </is>
       </c>
       <c r="C4">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4">
         <v>32</v>
@@ -23053,13 +23089,13 @@
         <v>2</v>
       </c>
       <c r="N4">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O4">
         <v>43</v>
       </c>
       <c r="P4">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -23105,7 +23141,7 @@
         <v>22</v>
       </c>
       <c r="N5">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="O5">
         <v>26</v>
@@ -23157,7 +23193,7 @@
         <v>24</v>
       </c>
       <c r="N6">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O6">
         <v>23</v>
@@ -23209,7 +23245,7 @@
         <v>18</v>
       </c>
       <c r="N7">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O7">
         <v>41</v>
@@ -23228,7 +23264,7 @@
         </is>
       </c>
       <c r="C8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D8">
         <v>19</v>
@@ -23329,7 +23365,7 @@
         </is>
       </c>
       <c r="C10">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D10">
         <v>38</v>
@@ -23362,7 +23398,7 @@
         <v>6</v>
       </c>
       <c r="N10">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O10">
         <v>39</v>
@@ -23466,7 +23502,7 @@
         <v>30</v>
       </c>
       <c r="N12">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O12">
         <v>38</v>
@@ -23518,7 +23554,7 @@
         <v>19</v>
       </c>
       <c r="N13">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O13">
         <v>11</v>
@@ -23622,7 +23658,7 @@
         <v>20</v>
       </c>
       <c r="N15">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="O15">
         <v>16</v>
@@ -23693,7 +23729,7 @@
         </is>
       </c>
       <c r="C17">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D17">
         <v>44</v>
@@ -23745,7 +23781,7 @@
         </is>
       </c>
       <c r="C18">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D18">
         <v>14</v>
@@ -23778,7 +23814,7 @@
         <v>33</v>
       </c>
       <c r="N18">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O18">
         <v>24</v>
@@ -23830,7 +23866,7 @@
         <v>44</v>
       </c>
       <c r="N19">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O19">
         <v>42</v>
@@ -23882,7 +23918,7 @@
         <v>47</v>
       </c>
       <c r="N20">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O20">
         <v>3</v>
@@ -23953,7 +23989,7 @@
         </is>
       </c>
       <c r="C22">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D22">
         <v>6</v>
@@ -24057,7 +24093,7 @@
         </is>
       </c>
       <c r="C24">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>25</v>
@@ -24142,10 +24178,10 @@
         <v>26</v>
       </c>
       <c r="N25">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O25">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P25">
         <v>43</v>
@@ -24161,7 +24197,7 @@
         </is>
       </c>
       <c r="C26">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D26">
         <v>4</v>
@@ -24194,7 +24230,7 @@
         <v>39</v>
       </c>
       <c r="N26">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O26">
         <v>31</v>
@@ -24213,7 +24249,7 @@
         </is>
       </c>
       <c r="C27">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D27">
         <v>18</v>
@@ -24246,10 +24282,10 @@
         <v>32</v>
       </c>
       <c r="N27">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="O27">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="P27">
         <v>40</v>
@@ -24298,7 +24334,7 @@
         <v>37</v>
       </c>
       <c r="N28">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="O28">
         <v>20</v>
@@ -24350,7 +24386,7 @@
         <v>1</v>
       </c>
       <c r="N29">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O29">
         <v>40</v>
@@ -24369,7 +24405,7 @@
         </is>
       </c>
       <c r="C30">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D30">
         <v>15</v>
@@ -24421,7 +24457,7 @@
         </is>
       </c>
       <c r="C31">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D31">
         <v>45</v>
@@ -24454,7 +24490,7 @@
         <v>25</v>
       </c>
       <c r="N31">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="O31">
         <v>17</v>
@@ -24506,10 +24542,10 @@
         <v>13</v>
       </c>
       <c r="N32">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O32">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="P32">
         <v>20</v>
@@ -24577,7 +24613,7 @@
         </is>
       </c>
       <c r="C34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D34">
         <v>3</v>
@@ -24610,7 +24646,7 @@
         <v>31</v>
       </c>
       <c r="N34">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="O34">
         <v>22</v>
@@ -24785,7 +24821,7 @@
         </is>
       </c>
       <c r="C38">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D38">
         <v>28</v>
@@ -24818,7 +24854,7 @@
         <v>15</v>
       </c>
       <c r="N38">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="O38">
         <v>34</v>
@@ -24941,7 +24977,7 @@
         </is>
       </c>
       <c r="C41">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D41">
         <v>1</v>
@@ -24974,10 +25010,10 @@
         <v>27</v>
       </c>
       <c r="N41">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O41">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P41">
         <v>45</v>
@@ -24993,7 +25029,7 @@
         </is>
       </c>
       <c r="C42">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D42">
         <v>34</v>
@@ -25026,7 +25062,7 @@
         <v>48</v>
       </c>
       <c r="N42">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O42">
         <v>5</v>
@@ -25045,7 +25081,7 @@
         </is>
       </c>
       <c r="C43">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="D43">
         <v>12</v>
@@ -25077,6 +25113,15 @@
       <c r="M43">
         <v>11</v>
       </c>
+      <c r="N43">
+        <v>22</v>
+      </c>
+      <c r="O43">
+        <v>46</v>
+      </c>
+      <c r="P43">
+        <v>48</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -25088,7 +25133,7 @@
         </is>
       </c>
       <c r="C44">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D44">
         <v>41</v>
@@ -25121,7 +25166,7 @@
         <v>3</v>
       </c>
       <c r="N44">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="O44">
         <v>33</v>
@@ -25173,7 +25218,7 @@
         <v>8</v>
       </c>
       <c r="N45">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O45">
         <v>7</v>
@@ -25244,7 +25289,7 @@
         </is>
       </c>
       <c r="C47">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D47">
         <v>2</v>
@@ -25277,7 +25322,7 @@
         <v>10</v>
       </c>
       <c r="N47">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="O47">
         <v>12</v>
@@ -25329,7 +25374,7 @@
         <v>23</v>
       </c>
       <c r="N48">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O48">
         <v>29</v>
@@ -25387,7 +25432,7 @@
         <v>44</v>
       </c>
       <c r="P49">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50">
@@ -25452,7 +25497,7 @@
         </is>
       </c>
       <c r="C51">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D51">
         <v>21</v>

</xml_diff>